<commit_message>
feat(admin+quality): panel de trazabilidad de casos, peso de reparto de Calidad y progreso de carga v5.30
- v5.30: fauchard_config.quality_reserved_case_weight para ponderar casos reservados en el round-robin de revisores de Calidad
- Nuevo panel admin de trazabilidad de casos (case-trace) para diagnóstico de estados/asignaciones
- Progreso de carga de archivos (uploadWithProgress) en creación/detalle de casos

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/Validación de Campos.xlsx
+++ b/docs/Validación de Campos.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/jaimecontreras/Documents/Projects/DentFlowAi/docs/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AE8FC2DC-D6FD-F246-BB9D-3817F10DC3E7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{69D7A674-9853-314E-A6E2-9C6DCF2DABAA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="33600" windowHeight="21000" xr2:uid="{26B86058-374B-8242-AB1D-7E59228E4242}"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="33600" windowHeight="21000" activeTab="1" xr2:uid="{26B86058-374B-8242-AB1D-7E59228E4242}"/>
   </bookViews>
   <sheets>
     <sheet name="Creación del Caso" sheetId="1" r:id="rId1"/>
@@ -487,9 +487,6 @@
     <t>Otro</t>
   </si>
   <si>
-    <t xml:space="preserve">La idea es completar la lista de precios en base a los campos que determinen el costo </t>
-  </si>
-  <si>
     <t>El costo es lo que se le pagará al técnico, y sobre eso se aplicará un % el cual debe cubrir gastos operacional y margen</t>
   </si>
   <si>
@@ -704,13 +701,26 @@
   </si>
   <si>
     <t>NO</t>
+  </si>
+  <si>
+    <t>La idea es completar la lista de precios en base a los campos que determinen el costo , los que están en la tabla u otros</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="3" x14ac:knownFonts="1">
+  <numFmts count="1">
+    <numFmt numFmtId="42" formatCode="_ &quot;$&quot;* #,##0_ ;_ &quot;$&quot;* \-#,##0_ ;_ &quot;$&quot;* &quot;-&quot;_ ;_ @_ "/>
+  </numFmts>
+  <fonts count="5" x14ac:knownFonts="1">
+    <font>
+      <sz val="12"/>
+      <color theme="1"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
     <font>
       <sz val="12"/>
       <color theme="1"/>
@@ -733,13 +743,26 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <b/>
+      <sz val="14"/>
+      <color theme="0"/>
+      <name val="Aptos Narrow"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="3" tint="0.499984740745262"/>
+        <bgColor indexed="64"/>
+      </patternFill>
     </fill>
   </fills>
   <borders count="1">
@@ -751,11 +774,12 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="2">
+  <cellStyleXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="11">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
@@ -769,21 +793,24 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="2" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="42" fontId="0" fillId="0" borderId="0" xfId="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
   </cellXfs>
-  <cellStyles count="2">
-    <cellStyle name="Hipervínculo" xfId="1" builtinId="8"/>
+  <cellStyles count="3">
+    <cellStyle name="Hipervínculo" xfId="2" builtinId="8"/>
+    <cellStyle name="Moneda [0]" xfId="1" builtinId="7"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="13">
@@ -890,7 +917,7 @@
     <tableColumn id="3" xr3:uid="{83D754FA-3A1B-154C-A888-BB7556C9D09C}" name="Urgencia"/>
     <tableColumn id="4" xr3:uid="{8400D6A7-4DD2-5043-A41C-D452813DA51D}" name="Material"/>
     <tableColumn id="5" xr3:uid="{0E30E7CA-560F-5E42-996B-5F6A45C9EF92}" name="Color"/>
-    <tableColumn id="6" xr3:uid="{70FBBE49-70D7-7041-BB13-7BFFCBDBCDD7}" name="Costo técnico (CLP)"/>
+    <tableColumn id="6" xr3:uid="{70FBBE49-70D7-7041-BB13-7BFFCBDBCDD7}" name="Costo técnico (CLP)" dataCellStyle="Moneda [0]"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleDark2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -1297,7 +1324,7 @@
         <v>4</v>
       </c>
       <c r="G1" s="3" t="s">
-        <v>214</v>
+        <v>213</v>
       </c>
       <c r="H1" s="3" t="s">
         <v>5</v>
@@ -1329,7 +1356,7 @@
         <v>4</v>
       </c>
       <c r="G2" s="3" t="s">
-        <v>219</v>
+        <v>218</v>
       </c>
       <c r="H2" s="2" t="s">
         <v>12</v>
@@ -1355,7 +1382,7 @@
         <v>4</v>
       </c>
       <c r="G3" s="3" t="s">
-        <v>219</v>
+        <v>218</v>
       </c>
       <c r="H3" s="2" t="s">
         <v>12</v>
@@ -1381,7 +1408,7 @@
         <v>4</v>
       </c>
       <c r="G4" s="8" t="s">
-        <v>215</v>
+        <v>214</v>
       </c>
       <c r="H4" s="2" t="s">
         <v>12</v>
@@ -1407,7 +1434,7 @@
         <v>4</v>
       </c>
       <c r="G5" s="3" t="s">
-        <v>219</v>
+        <v>218</v>
       </c>
       <c r="H5" s="2" t="s">
         <v>12</v>
@@ -1433,7 +1460,7 @@
         <v>4</v>
       </c>
       <c r="G6" s="3" t="s">
-        <v>219</v>
+        <v>218</v>
       </c>
       <c r="H6" s="2" t="s">
         <v>12</v>
@@ -1459,7 +1486,7 @@
         <v>4</v>
       </c>
       <c r="G7" s="8" t="s">
-        <v>215</v>
+        <v>214</v>
       </c>
       <c r="H7" s="2" t="s">
         <v>12</v>
@@ -1485,7 +1512,7 @@
         <v>4</v>
       </c>
       <c r="G8" s="8" t="s">
-        <v>215</v>
+        <v>214</v>
       </c>
       <c r="H8" s="2" t="s">
         <v>12</v>
@@ -1511,7 +1538,7 @@
         <v>4</v>
       </c>
       <c r="G9" s="3" t="s">
-        <v>219</v>
+        <v>218</v>
       </c>
       <c r="H9" s="2" t="s">
         <v>12</v>
@@ -1537,7 +1564,7 @@
         <v>38</v>
       </c>
       <c r="G10" s="3" t="s">
-        <v>219</v>
+        <v>218</v>
       </c>
       <c r="H10" s="2" t="s">
         <v>129</v>
@@ -1563,7 +1590,7 @@
         <v>42</v>
       </c>
       <c r="G11" s="3" t="s">
-        <v>219</v>
+        <v>218</v>
       </c>
       <c r="H11" s="2" t="s">
         <v>129</v>
@@ -1589,7 +1616,7 @@
         <v>4</v>
       </c>
       <c r="G12" s="8" t="s">
-        <v>215</v>
+        <v>214</v>
       </c>
       <c r="H12" s="2" t="s">
         <v>12</v>
@@ -1615,7 +1642,7 @@
         <v>64</v>
       </c>
       <c r="G13" s="3" t="s">
-        <v>219</v>
+        <v>218</v>
       </c>
       <c r="H13" s="2" t="s">
         <v>129</v>
@@ -1641,7 +1668,7 @@
         <v>4</v>
       </c>
       <c r="G14" s="3" t="s">
-        <v>219</v>
+        <v>218</v>
       </c>
       <c r="H14" s="2" t="s">
         <v>12</v>
@@ -1667,7 +1694,7 @@
         <v>4</v>
       </c>
       <c r="G15" s="3" t="s">
-        <v>219</v>
+        <v>218</v>
       </c>
       <c r="H15" s="2" t="s">
         <v>57</v>
@@ -1693,7 +1720,7 @@
         <v>4</v>
       </c>
       <c r="G16" s="3" t="s">
-        <v>219</v>
+        <v>218</v>
       </c>
       <c r="H16" s="2" t="s">
         <v>129</v>
@@ -1719,7 +1746,7 @@
         <v>4</v>
       </c>
       <c r="G17" s="3" t="s">
-        <v>219</v>
+        <v>218</v>
       </c>
       <c r="H17" s="2" t="s">
         <v>64</v>
@@ -1745,7 +1772,7 @@
         <v>68</v>
       </c>
       <c r="G18" s="3" t="s">
-        <v>219</v>
+        <v>218</v>
       </c>
       <c r="H18" s="2" t="s">
         <v>129</v>
@@ -1771,7 +1798,7 @@
         <v>64</v>
       </c>
       <c r="G19" s="3" t="s">
-        <v>219</v>
+        <v>218</v>
       </c>
       <c r="H19" s="2" t="s">
         <v>12</v>
@@ -1797,7 +1824,7 @@
         <v>64</v>
       </c>
       <c r="G20" s="3" t="s">
-        <v>219</v>
+        <v>218</v>
       </c>
       <c r="H20" s="2" t="s">
         <v>129</v>
@@ -1823,7 +1850,7 @@
         <v>64</v>
       </c>
       <c r="G21" s="3" t="s">
-        <v>219</v>
+        <v>218</v>
       </c>
       <c r="H21" s="2" t="s">
         <v>12</v>
@@ -1849,7 +1876,7 @@
         <v>64</v>
       </c>
       <c r="G22" s="3" t="s">
-        <v>219</v>
+        <v>218</v>
       </c>
       <c r="H22" s="2" t="s">
         <v>12</v>
@@ -1875,7 +1902,7 @@
         <v>64</v>
       </c>
       <c r="G23" s="3" t="s">
-        <v>219</v>
+        <v>218</v>
       </c>
       <c r="H23" s="2" t="s">
         <v>12</v>
@@ -1901,7 +1928,7 @@
         <v>64</v>
       </c>
       <c r="G24" s="3" t="s">
-        <v>219</v>
+        <v>218</v>
       </c>
       <c r="H24" s="2" t="s">
         <v>129</v>
@@ -1927,7 +1954,7 @@
         <v>64</v>
       </c>
       <c r="G25" s="3" t="s">
-        <v>219</v>
+        <v>218</v>
       </c>
       <c r="H25" s="2" t="s">
         <v>129</v>
@@ -1953,7 +1980,7 @@
         <v>64</v>
       </c>
       <c r="G26" s="3" t="s">
-        <v>219</v>
+        <v>218</v>
       </c>
       <c r="H26" s="2" t="s">
         <v>12</v>
@@ -1979,7 +2006,7 @@
         <v>64</v>
       </c>
       <c r="G27" s="3" t="s">
-        <v>219</v>
+        <v>218</v>
       </c>
       <c r="H27" s="2" t="s">
         <v>129</v>
@@ -2005,7 +2032,7 @@
         <v>64</v>
       </c>
       <c r="G28" s="3" t="s">
-        <v>219</v>
+        <v>218</v>
       </c>
       <c r="H28" s="2" t="s">
         <v>129</v>
@@ -2027,13 +2054,14 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6CB2E25B-228F-574D-846D-957A01619C29}">
-  <dimension ref="A1:J28"/>
+  <dimension ref="A1:J29"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="2" max="2" width="19.6640625" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="13" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="10.6640625" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="22.6640625" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="118.1640625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:10" x14ac:dyDescent="0.2">
@@ -2073,11 +2101,11 @@
       <c r="E2" t="s">
         <v>136</v>
       </c>
-      <c r="J2" t="s">
-        <v>147</v>
-      </c>
-    </row>
-    <row r="3" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="F2" s="9">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="3" spans="1:10" ht="19" x14ac:dyDescent="0.25">
       <c r="A3">
         <v>2</v>
       </c>
@@ -2093,11 +2121,14 @@
       <c r="E3" t="s">
         <v>136</v>
       </c>
-      <c r="J3" t="s">
-        <v>148</v>
-      </c>
-    </row>
-    <row r="4" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="F3" s="9">
+        <v>0</v>
+      </c>
+      <c r="J3" s="10" t="s">
+        <v>147</v>
+      </c>
+    </row>
+    <row r="4" spans="1:10" ht="19" x14ac:dyDescent="0.25">
       <c r="A4">
         <v>3</v>
       </c>
@@ -2112,6 +2143,12 @@
       </c>
       <c r="E4" t="s">
         <v>136</v>
+      </c>
+      <c r="F4" s="9">
+        <v>0</v>
+      </c>
+      <c r="J4" s="10" t="s">
+        <v>219</v>
       </c>
     </row>
     <row r="5" spans="1:10" x14ac:dyDescent="0.2">
@@ -2130,6 +2167,9 @@
       <c r="E5" t="s">
         <v>136</v>
       </c>
+      <c r="F5" s="9">
+        <v>0</v>
+      </c>
     </row>
     <row r="6" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A6">
@@ -2147,6 +2187,9 @@
       <c r="E6" t="s">
         <v>136</v>
       </c>
+      <c r="F6" s="9">
+        <v>0</v>
+      </c>
     </row>
     <row r="7" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A7">
@@ -2164,6 +2207,9 @@
       <c r="E7" t="s">
         <v>136</v>
       </c>
+      <c r="F7" s="9">
+        <v>0</v>
+      </c>
     </row>
     <row r="8" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A8">
@@ -2181,6 +2227,9 @@
       <c r="E8" t="s">
         <v>136</v>
       </c>
+      <c r="F8" s="9">
+        <v>0</v>
+      </c>
     </row>
     <row r="9" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A9">
@@ -2198,6 +2247,9 @@
       <c r="E9" t="s">
         <v>136</v>
       </c>
+      <c r="F9" s="9">
+        <v>0</v>
+      </c>
     </row>
     <row r="10" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A10">
@@ -2215,6 +2267,9 @@
       <c r="E10" t="s">
         <v>136</v>
       </c>
+      <c r="F10" s="9">
+        <v>0</v>
+      </c>
     </row>
     <row r="11" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A11">
@@ -2232,6 +2287,9 @@
       <c r="E11" t="s">
         <v>136</v>
       </c>
+      <c r="F11" s="9">
+        <v>0</v>
+      </c>
     </row>
     <row r="12" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A12">
@@ -2249,6 +2307,9 @@
       <c r="E12" t="s">
         <v>136</v>
       </c>
+      <c r="F12" s="9">
+        <v>0</v>
+      </c>
     </row>
     <row r="13" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A13">
@@ -2266,6 +2327,9 @@
       <c r="E13" t="s">
         <v>136</v>
       </c>
+      <c r="F13" s="9">
+        <v>0</v>
+      </c>
     </row>
     <row r="14" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A14">
@@ -2283,6 +2347,9 @@
       <c r="E14" t="s">
         <v>136</v>
       </c>
+      <c r="F14" s="9">
+        <v>0</v>
+      </c>
     </row>
     <row r="15" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A15">
@@ -2300,6 +2367,9 @@
       <c r="E15" t="s">
         <v>136</v>
       </c>
+      <c r="F15" s="9">
+        <v>0</v>
+      </c>
     </row>
     <row r="16" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A16">
@@ -2317,8 +2387,11 @@
       <c r="E16" t="s">
         <v>136</v>
       </c>
-    </row>
-    <row r="17" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="F16" s="9">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="17" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A17">
         <v>16</v>
       </c>
@@ -2334,8 +2407,11 @@
       <c r="E17" t="s">
         <v>136</v>
       </c>
-    </row>
-    <row r="18" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="F17" s="9">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="18" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A18">
         <v>17</v>
       </c>
@@ -2351,8 +2427,11 @@
       <c r="E18" t="s">
         <v>136</v>
       </c>
-    </row>
-    <row r="19" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="F18" s="9">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="19" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A19">
         <v>18</v>
       </c>
@@ -2368,8 +2447,11 @@
       <c r="E19" t="s">
         <v>136</v>
       </c>
-    </row>
-    <row r="20" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="F19" s="9">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="20" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A20">
         <v>19</v>
       </c>
@@ -2385,8 +2467,11 @@
       <c r="E20" t="s">
         <v>136</v>
       </c>
-    </row>
-    <row r="21" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="F20" s="9">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="21" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A21">
         <v>20</v>
       </c>
@@ -2402,8 +2487,11 @@
       <c r="E21" t="s">
         <v>136</v>
       </c>
-    </row>
-    <row r="22" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="F21" s="9">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="22" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A22">
         <v>21</v>
       </c>
@@ -2419,8 +2507,11 @@
       <c r="E22" t="s">
         <v>136</v>
       </c>
-    </row>
-    <row r="23" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="F22" s="9">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="23" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A23">
         <v>22</v>
       </c>
@@ -2436,8 +2527,11 @@
       <c r="E23" t="s">
         <v>136</v>
       </c>
-    </row>
-    <row r="24" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="F23" s="9">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="24" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A24">
         <v>23</v>
       </c>
@@ -2453,8 +2547,11 @@
       <c r="E24" t="s">
         <v>136</v>
       </c>
-    </row>
-    <row r="25" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="F24" s="9">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="25" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A25">
         <v>24</v>
       </c>
@@ -2470,8 +2567,11 @@
       <c r="E25" t="s">
         <v>136</v>
       </c>
-    </row>
-    <row r="26" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="F25" s="9">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="26" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A26">
         <v>25</v>
       </c>
@@ -2487,8 +2587,11 @@
       <c r="E26" t="s">
         <v>136</v>
       </c>
-    </row>
-    <row r="27" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="F26" s="9">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="27" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A27">
         <v>26</v>
       </c>
@@ -2504,8 +2607,11 @@
       <c r="E27" t="s">
         <v>136</v>
       </c>
-    </row>
-    <row r="28" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="F27" s="9">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="28" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A28">
         <v>27</v>
       </c>
@@ -2521,6 +2627,12 @@
       <c r="E28" t="s">
         <v>136</v>
       </c>
+      <c r="F28" s="9">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="29" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="F29" s="9"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -2540,10 +2652,10 @@
         <v>130</v>
       </c>
       <c r="B1" t="s">
+        <v>148</v>
+      </c>
+      <c r="C1" t="s">
         <v>149</v>
-      </c>
-      <c r="C1" t="s">
-        <v>150</v>
       </c>
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.2">
@@ -2551,7 +2663,7 @@
         <v>1</v>
       </c>
       <c r="B2" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
       <c r="C2" t="s">
         <v>134</v>
@@ -2562,7 +2674,7 @@
         <v>2</v>
       </c>
       <c r="B3" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
       <c r="C3" t="s">
         <v>139</v>
@@ -2573,7 +2685,7 @@
         <v>3</v>
       </c>
       <c r="B4" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
       <c r="C4" t="s">
         <v>140</v>
@@ -2584,7 +2696,7 @@
         <v>4</v>
       </c>
       <c r="B5" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="C5" t="s">
         <v>141</v>
@@ -2595,7 +2707,7 @@
         <v>5</v>
       </c>
       <c r="B6" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="C6" t="s">
         <v>142</v>
@@ -2606,7 +2718,7 @@
         <v>6</v>
       </c>
       <c r="B7" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="C7" t="s">
         <v>143</v>
@@ -2617,7 +2729,7 @@
         <v>7</v>
       </c>
       <c r="B8" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="C8" t="s">
         <v>144</v>
@@ -2628,7 +2740,7 @@
         <v>8</v>
       </c>
       <c r="B9" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="C9" t="s">
         <v>145</v>
@@ -2639,7 +2751,7 @@
         <v>9</v>
       </c>
       <c r="B10" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="C10" t="s">
         <v>146</v>
@@ -2663,10 +2775,10 @@
         <v>130</v>
       </c>
       <c r="B1" t="s">
+        <v>148</v>
+      </c>
+      <c r="C1" t="s">
         <v>149</v>
-      </c>
-      <c r="C1" t="s">
-        <v>150</v>
       </c>
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.2">
@@ -2674,7 +2786,7 @@
         <v>1</v>
       </c>
       <c r="B2" t="s">
-        <v>216</v>
+        <v>215</v>
       </c>
       <c r="C2" t="s">
         <v>135</v>
@@ -2685,7 +2797,7 @@
         <v>2</v>
       </c>
       <c r="B3" t="s">
-        <v>217</v>
+        <v>216</v>
       </c>
       <c r="C3" t="s">
         <v>137</v>
@@ -2696,7 +2808,7 @@
         <v>3</v>
       </c>
       <c r="B4" t="s">
-        <v>218</v>
+        <v>217</v>
       </c>
       <c r="C4" t="s">
         <v>138</v>
@@ -2725,10 +2837,10 @@
         <v>130</v>
       </c>
       <c r="B1" t="s">
+        <v>148</v>
+      </c>
+      <c r="C1" t="s">
         <v>149</v>
-      </c>
-      <c r="C1" t="s">
-        <v>150</v>
       </c>
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.2">
@@ -2736,10 +2848,10 @@
         <v>1</v>
       </c>
       <c r="B2" t="s">
+        <v>159</v>
+      </c>
+      <c r="C2" t="s">
         <v>160</v>
-      </c>
-      <c r="C2" t="s">
-        <v>161</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.2">
@@ -2747,10 +2859,10 @@
         <v>2</v>
       </c>
       <c r="B3" t="s">
+        <v>161</v>
+      </c>
+      <c r="C3" t="s">
         <v>162</v>
-      </c>
-      <c r="C3" t="s">
-        <v>163</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.2">
@@ -2758,10 +2870,10 @@
         <v>3</v>
       </c>
       <c r="B4" t="s">
+        <v>163</v>
+      </c>
+      <c r="C4" t="s">
         <v>164</v>
-      </c>
-      <c r="C4" t="s">
-        <v>165</v>
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.2">
@@ -2769,10 +2881,10 @@
         <v>4</v>
       </c>
       <c r="B5" t="s">
+        <v>165</v>
+      </c>
+      <c r="C5" t="s">
         <v>166</v>
-      </c>
-      <c r="C5" t="s">
-        <v>167</v>
       </c>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.2">
@@ -2780,10 +2892,10 @@
         <v>5</v>
       </c>
       <c r="B6" t="s">
+        <v>167</v>
+      </c>
+      <c r="C6" t="s">
         <v>168</v>
-      </c>
-      <c r="C6" t="s">
-        <v>169</v>
       </c>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.2">
@@ -2791,10 +2903,10 @@
         <v>6</v>
       </c>
       <c r="B7" t="s">
+        <v>169</v>
+      </c>
+      <c r="C7" t="s">
         <v>170</v>
-      </c>
-      <c r="C7" t="s">
-        <v>171</v>
       </c>
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.2">
@@ -2802,10 +2914,10 @@
         <v>7</v>
       </c>
       <c r="B8" t="s">
+        <v>171</v>
+      </c>
+      <c r="C8" t="s">
         <v>172</v>
-      </c>
-      <c r="C8" t="s">
-        <v>173</v>
       </c>
     </row>
     <row r="9" spans="1:3" x14ac:dyDescent="0.2">
@@ -2813,10 +2925,10 @@
         <v>8</v>
       </c>
       <c r="B9" t="s">
+        <v>173</v>
+      </c>
+      <c r="C9" t="s">
         <v>174</v>
-      </c>
-      <c r="C9" t="s">
-        <v>175</v>
       </c>
     </row>
     <row r="10" spans="1:3" x14ac:dyDescent="0.2">
@@ -2824,10 +2936,10 @@
         <v>9</v>
       </c>
       <c r="B10" t="s">
+        <v>175</v>
+      </c>
+      <c r="C10" t="s">
         <v>176</v>
-      </c>
-      <c r="C10" t="s">
-        <v>177</v>
       </c>
     </row>
     <row r="11" spans="1:3" x14ac:dyDescent="0.2">
@@ -2835,10 +2947,10 @@
         <v>10</v>
       </c>
       <c r="B11" t="s">
+        <v>177</v>
+      </c>
+      <c r="C11" t="s">
         <v>178</v>
-      </c>
-      <c r="C11" t="s">
-        <v>179</v>
       </c>
     </row>
     <row r="12" spans="1:3" x14ac:dyDescent="0.2">
@@ -2846,7 +2958,7 @@
         <v>11</v>
       </c>
       <c r="B12" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
       <c r="C12" t="s">
         <v>146</v>
@@ -2875,10 +2987,10 @@
         <v>130</v>
       </c>
       <c r="B1" t="s">
+        <v>148</v>
+      </c>
+      <c r="C1" t="s">
         <v>149</v>
-      </c>
-      <c r="C1" t="s">
-        <v>150</v>
       </c>
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.2">
@@ -2886,10 +2998,10 @@
         <v>1</v>
       </c>
       <c r="B2" t="s">
+        <v>180</v>
+      </c>
+      <c r="C2" t="s">
         <v>181</v>
-      </c>
-      <c r="C2" t="s">
-        <v>182</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.2">
@@ -2897,10 +3009,10 @@
         <v>2</v>
       </c>
       <c r="B3" t="s">
+        <v>182</v>
+      </c>
+      <c r="C3" t="s">
         <v>183</v>
-      </c>
-      <c r="C3" t="s">
-        <v>184</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.2">
@@ -2908,10 +3020,10 @@
         <v>3</v>
       </c>
       <c r="B4" t="s">
+        <v>184</v>
+      </c>
+      <c r="C4" t="s">
         <v>185</v>
-      </c>
-      <c r="C4" t="s">
-        <v>186</v>
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.2">
@@ -2919,10 +3031,10 @@
         <v>4</v>
       </c>
       <c r="B5" t="s">
+        <v>186</v>
+      </c>
+      <c r="C5" t="s">
         <v>187</v>
-      </c>
-      <c r="C5" t="s">
-        <v>188</v>
       </c>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.2">
@@ -2930,10 +3042,10 @@
         <v>5</v>
       </c>
       <c r="B6" t="s">
+        <v>188</v>
+      </c>
+      <c r="C6" t="s">
         <v>189</v>
-      </c>
-      <c r="C6" t="s">
-        <v>190</v>
       </c>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.2">
@@ -2941,10 +3053,10 @@
         <v>6</v>
       </c>
       <c r="B7" t="s">
+        <v>190</v>
+      </c>
+      <c r="C7" t="s">
         <v>191</v>
-      </c>
-      <c r="C7" t="s">
-        <v>192</v>
       </c>
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.2">
@@ -2952,10 +3064,10 @@
         <v>7</v>
       </c>
       <c r="B8" t="s">
+        <v>192</v>
+      </c>
+      <c r="C8" t="s">
         <v>193</v>
-      </c>
-      <c r="C8" t="s">
-        <v>194</v>
       </c>
     </row>
     <row r="9" spans="1:3" x14ac:dyDescent="0.2">
@@ -2963,10 +3075,10 @@
         <v>8</v>
       </c>
       <c r="B9" t="s">
+        <v>194</v>
+      </c>
+      <c r="C9" t="s">
         <v>195</v>
-      </c>
-      <c r="C9" t="s">
-        <v>196</v>
       </c>
     </row>
     <row r="10" spans="1:3" x14ac:dyDescent="0.2">
@@ -2974,10 +3086,10 @@
         <v>9</v>
       </c>
       <c r="B10" t="s">
+        <v>196</v>
+      </c>
+      <c r="C10" t="s">
         <v>197</v>
-      </c>
-      <c r="C10" t="s">
-        <v>198</v>
       </c>
     </row>
     <row r="11" spans="1:3" x14ac:dyDescent="0.2">
@@ -2985,10 +3097,10 @@
         <v>10</v>
       </c>
       <c r="B11" t="s">
+        <v>198</v>
+      </c>
+      <c r="C11" t="s">
         <v>199</v>
-      </c>
-      <c r="C11" t="s">
-        <v>200</v>
       </c>
     </row>
     <row r="12" spans="1:3" x14ac:dyDescent="0.2">
@@ -2996,10 +3108,10 @@
         <v>11</v>
       </c>
       <c r="B12" t="s">
+        <v>200</v>
+      </c>
+      <c r="C12" t="s">
         <v>201</v>
-      </c>
-      <c r="C12" t="s">
-        <v>202</v>
       </c>
     </row>
     <row r="13" spans="1:3" x14ac:dyDescent="0.2">
@@ -3007,10 +3119,10 @@
         <v>12</v>
       </c>
       <c r="B13" t="s">
+        <v>202</v>
+      </c>
+      <c r="C13" t="s">
         <v>203</v>
-      </c>
-      <c r="C13" t="s">
-        <v>204</v>
       </c>
     </row>
     <row r="14" spans="1:3" x14ac:dyDescent="0.2">
@@ -3018,10 +3130,10 @@
         <v>13</v>
       </c>
       <c r="B14" t="s">
+        <v>204</v>
+      </c>
+      <c r="C14" t="s">
         <v>205</v>
-      </c>
-      <c r="C14" t="s">
-        <v>206</v>
       </c>
     </row>
     <row r="15" spans="1:3" x14ac:dyDescent="0.2">
@@ -3029,10 +3141,10 @@
         <v>14</v>
       </c>
       <c r="B15" t="s">
+        <v>206</v>
+      </c>
+      <c r="C15" t="s">
         <v>207</v>
-      </c>
-      <c r="C15" t="s">
-        <v>208</v>
       </c>
     </row>
     <row r="16" spans="1:3" x14ac:dyDescent="0.2">
@@ -3040,10 +3152,10 @@
         <v>15</v>
       </c>
       <c r="B16" t="s">
+        <v>208</v>
+      </c>
+      <c r="C16" t="s">
         <v>209</v>
-      </c>
-      <c r="C16" t="s">
-        <v>210</v>
       </c>
     </row>
     <row r="17" spans="1:3" x14ac:dyDescent="0.2">
@@ -3051,10 +3163,10 @@
         <v>16</v>
       </c>
       <c r="B17" t="s">
+        <v>210</v>
+      </c>
+      <c r="C17" t="s">
         <v>211</v>
-      </c>
-      <c r="C17" t="s">
-        <v>212</v>
       </c>
     </row>
     <row r="18" spans="1:3" x14ac:dyDescent="0.2">
@@ -3062,7 +3174,7 @@
         <v>17</v>
       </c>
       <c r="B18" t="s">
-        <v>213</v>
+        <v>212</v>
       </c>
       <c r="C18" t="s">
         <v>146</v>

</xml_diff>